<commit_message>
Add documentation and CLI support for PDF extractor
  - Add comprehensive README with installation and usage instructions
  - Update main.py to accept PDF path as command line argument
  - Document project structure and dependencies
</commit_message>
<xml_diff>
--- a/data/output/invoice_data.xlsx
+++ b/data/output/invoice_data.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Invoice Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invoice Data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Commit for file extraction and login logic
</commit_message>
<xml_diff>
--- a/data/output/invoice_data.xlsx
+++ b/data/output/invoice_data.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invoice Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Invoice Data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,20 +413,130 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Company Name</t>
+          <t>Invoice Number</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Invoice Date</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Mode / Terms of Payment</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Seller Name</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Buyer Name</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Buyer Mobile</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Product / Model</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>State Code</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>OEM / Description</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Total Invoice Amount</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Item Code</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>SALE-CR-2573</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>29-Dec-25</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Google Pay Account</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>Msg technologies 2025-2026</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>S.DEEPANKUMAR</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>9790321415</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>SWIFT</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Tamil Nadu</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>165/80 R14 BRIDGESTONE S248 T</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>16,400.00</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>40111010</t>
         </is>
       </c>
     </row>

</xml_diff>